<commit_message>
updated openai predictions scripts
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/buildings/112301/features.xlsx
+++ b/buildings/112301/features.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BJ2"/>
+  <dimension ref="A1:BD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,250 +491,220 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>SCHADSTOFF</t>
+          <t>FASSADE_BEKLEIDUNG</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>SCHADSTOFF_confidence</t>
+          <t>FASSADE_BEKLEIDUNG_confidence</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>KONSTRUKTION_DACH</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>KONSTRUKTION_DACH_confidence</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>DACH_BEKLEIDUNG</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>DACH_BEKLEIDUNG_confidence</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>PHOTOVOLTAIK</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PHOTOVOLTAIK_confidence</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>FENSTER</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>FENSTER_confidence</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>HOLZ</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>HOLZ_confidence</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>BETON</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>BETON_confidence</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>STAHL</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>STAHL_confidence</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>STAHLBLECH</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>STAHLBLECH_confidence</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>ETERNIT</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>ETERNIT_confidence</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>STEINPLATTEN</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>STEINPLATTEN_confidence</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>DACHZIEGEL</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>DACHZIEGEL_confidence</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>SPEZIELL</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>SPEZIELL_confidence</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>EXTRA</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>EXTRA_confidence</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>OVERALL_CONFIDENCE_PCT</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
           <t>TRAGWERK_FASSADE</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>TRAGWERK_FASSADE_confidence</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>FASSADE_DAEMMUNG</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>FASSADE_DAEMMUNG_confidence</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>FASSADE_BEKLEIDUNG</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>FASSADE_BEKLEIDUNG_confidence</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>KONSTRUKTION_DECKE</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>KONSTRUKTION_DECKE_confidence</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>BODENAUFBAU</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>BODENAUFBAU_confidence</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>KONSTRUKTION_DACH</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>KONSTRUKTION_DACH_confidence</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>DACH_BEKLEIDUNG</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>DACH_BEKLEIDUNG_confidence</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>PHOTOVOLTAIK</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>PHOTOVOLTAIK_confidence</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>FENSTER</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>FENSTER_confidence</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>HOLZ</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>HOLZ_confidence</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>BETON</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>BETON_confidence</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>STAHL</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>STAHL_confidence</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>STAHLBLECH</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>STAHLBLECH_confidence</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>ETERNIT</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>ETERNIT_confidence</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>STEINPLATTEN</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>STEINPLATTEN_confidence</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>DACHZIEGEL</t>
-        </is>
-      </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>DACHZIEGEL_confidence</t>
+          <t>PV_FLAECHE</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>SPEZIELL</t>
+          <t>FENSTERANZAHL</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>SPEZIELL_confidence</t>
+          <t>DAEMMUNGSFLAECHE</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>EXTRA</t>
+          <t>STAHL_LM</t>
         </is>
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>EXTRA_confidence</t>
+          <t>STAHLBLECH_FLAECHE</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>OVERALL_CONFIDENCE_PCT</t>
+          <t>ETERNIT_FLAECHE</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>PV_FLAECHE</t>
+          <t>STEINPLATTEN_FLAECHE</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>FENSTERANZAHL</t>
+          <t>DACHZIEGEL_FLAECHE</t>
         </is>
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>DAEMMUNGSFLAECHE</t>
+          <t>BETON_FLAECHE</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
         <is>
-          <t>STAHL_LM</t>
+          <t>HOLZ_LM</t>
         </is>
       </c>
       <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>STAHLBLECH_FLAECHE</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>ETERNIT_FLAECHE</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>STEINPLATTEN_FLAECHE</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>DACHZIEGEL_FLAECHE</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>BETON_FLAECHE</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>HOLZ_LM</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>HOLZ_FLAECHE</t>
         </is>
@@ -793,170 +763,134 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>LEICHTBAU HOLZPLATTEN, MIT UNTERKONSTRUKTION</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>STEILDACH, HOLZKONSTRUKTION</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ZIEGEL</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>AB 1990</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
           <t>UNBEKANNT</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>MASSIVBAU</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AH2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AK2" t="inlineStr">
         <is>
           <t>UNBEKANNT</t>
         </is>
       </c>
-      <c r="R2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>LEICHTBAU HOLZPLATTEN, MIT UNTERKONSTRUKTION</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="AL2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AM2" t="inlineStr">
         <is>
           <t>UNBEKANNT</t>
         </is>
       </c>
-      <c r="V2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>UNBEKANNT</t>
-        </is>
-      </c>
-      <c r="X2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>STEILDACH, HOLZKONSTRUKTION</t>
-        </is>
-      </c>
-      <c r="Z2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>ZIEGEL</t>
-        </is>
-      </c>
-      <c r="AB2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>AB 1990</t>
-        </is>
-      </c>
-      <c r="AF2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="AH2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>UNKLAR</t>
-        </is>
-      </c>
-      <c r="AL2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
       <c r="AN2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AP2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AR2" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="AT2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>UNKLAR</t>
-        </is>
-      </c>
-      <c r="AV2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>UNKLAR</t>
-        </is>
-      </c>
-      <c r="AX2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>55.3</v>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="inlineStr"/>
       <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
       <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
updated UI, added new images instead of iframe
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/buildings/112301/features.xlsx
+++ b/buildings/112301/features.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD2"/>
+  <dimension ref="A1:BE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,220 +491,225 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>ZH_MAP_URL</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>FASSADE_BEKLEIDUNG</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>FASSADE_BEKLEIDUNG_confidence</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>KONSTRUKTION_DACH</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>KONSTRUKTION_DACH_confidence</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DACH_BEKLEIDUNG</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>DACH_BEKLEIDUNG_confidence</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>PHOTOVOLTAIK</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PHOTOVOLTAIK_confidence</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>FENSTER</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>FENSTER_confidence</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>HOLZ</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>HOLZ_confidence</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>BETON</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>BETON_confidence</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>STAHL</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>STAHL_confidence</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>STAHLBLECH</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>STAHLBLECH_confidence</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>ETERNIT</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>ETERNIT_confidence</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>STEINPLATTEN</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>STEINPLATTEN_confidence</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>DACHZIEGEL</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>DACHZIEGEL_confidence</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>SPEZIELL</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>SPEZIELL_confidence</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>EXTRA</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>EXTRA_confidence</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>OVERALL_CONFIDENCE_PCT</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>TRAGWERK_FASSADE</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>FASSADE_DAEMMUNG</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>KONSTRUKTION_DECKE</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>BODENAUFBAU</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>PV_FLAECHE</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>FENSTERANZAHL</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>DAEMMUNGSFLAECHE</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>STAHL_LM</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>STAHLBLECH_FLAECHE</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>ETERNIT_FLAECHE</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>STEINPLATTEN_FLAECHE</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>DACHZIEGEL_FLAECHE</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>BETON_FLAECHE</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>HOLZ_LM</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>HOLZ_FLAECHE</t>
         </is>
@@ -763,120 +768,124 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>https://geo.zh.ch/maps?x=2705815&amp;y=1255933&amp;scale=900&amp;basemap=areavbackgroundzh</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>LEICHTBAU HOLZPLATTEN, MIT UNTERKONSTRUKTION</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>0.9</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>STEILDACH, HOLZKONSTRUKTION</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.7</v>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>ZIEGEL</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>UNBEKANNT</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>AB 1990</t>
+        </is>
+      </c>
+      <c r="W2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
         <v>0.8</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>UNKLAR</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>UNBEKANNT</t>
+        </is>
+      </c>
+      <c r="AG2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>JA</t>
         </is>
       </c>
-      <c r="T2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>AB 1990</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
+      <c r="AK2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>NEIN</t>
+        </is>
+      </c>
+      <c r="AM2" t="n">
         <v>0.5</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="X2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>NEIN</t>
         </is>
       </c>
-      <c r="Z2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>UNBEKANNT</t>
-        </is>
-      </c>
-      <c r="AB2" t="n">
+      <c r="AO2" t="n">
         <v>0.3</v>
       </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AF2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>NEIN</t>
-        </is>
-      </c>
-      <c r="AH2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>UNBEKANNT</t>
-        </is>
-      </c>
-      <c r="AL2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>UNBEKANNT</t>
-        </is>
-      </c>
-      <c r="AN2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>55.7</v>
-      </c>
-      <c r="AP2" t="inlineStr"/>
+      <c r="AP2" t="n">
+        <v>55</v>
+      </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
@@ -891,6 +900,7 @@
       <c r="BB2" t="inlineStr"/>
       <c r="BC2" t="inlineStr"/>
       <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>